<commit_message>
feat: actualizar datos de la Junta Directiva 2026-2028 presidida por Dr. José Eduardo Carvajal Obando
</commit_message>
<xml_diff>
--- a/Directorio_ARCCPCE_Oficial.xlsx
+++ b/Directorio_ARCCPCE_Oficial.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="D2" s="17" t="inlineStr">
         <is>
-          <t>Presidente Fundacional / Convocante</t>
+          <t>Presidente de la Junta Directiva (2026-2028)</t>
         </is>
       </c>
       <c r="E2" s="17" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="I2" s="16" t="inlineStr">
         <is>
-          <t>Socio Fundador Oficial</t>
+          <t>Activo - Junta Directiva (2026-2028)</t>
         </is>
       </c>
       <c r="J2" s="17" t="inlineStr">

</xml_diff>

<commit_message>
feat: incorporar seccion de Mesa Directiva Oficial 2026-2028 con fotografia oficial y actualizacion de Excel
</commit_message>
<xml_diff>
--- a/Directorio_ARCCPCE_Oficial.xlsx
+++ b/Directorio_ARCCPCE_Oficial.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directorio_Agremiados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones_Tecnicas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entidades_Alianzas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mesa_Directiva_2026_2028" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directorio_Agremiados" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones_Tecnicas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entidades_Alianzas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52,7 +53,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -99,6 +100,12 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F7FF"/>
+        <bgColor rgb="00F0F7FF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -140,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -203,6 +210,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -570,6 +592,325 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="51" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>Cargo en Mesa Directiva</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="inlineStr">
+        <is>
+          <t>Nombre Completo</t>
+        </is>
+      </c>
+      <c r="C1" s="22" t="inlineStr">
+        <is>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="D1" s="22" t="inlineStr">
+        <is>
+          <t>Grado Académico</t>
+        </is>
+      </c>
+      <c r="E1" s="22" t="inlineStr">
+        <is>
+          <t>País / Sede</t>
+        </is>
+      </c>
+      <c r="F1" s="22" t="inlineStr">
+        <is>
+          <t>Órgano / Comisión Técnica Asignada</t>
+        </is>
+      </c>
+      <c r="G1" s="22" t="inlineStr">
+        <is>
+          <t>Estado Institucional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Presidente</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>Dr. José Eduardo Carvajal Obando</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
+        <is>
+          <t>2026 – 2028</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>Doctor en Salud Pública / Especialista</t>
+        </is>
+      </c>
+      <c r="E2" s="25" t="inlineStr">
+        <is>
+          <t>Costa Rica (Sede Central)</t>
+        </is>
+      </c>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>Junta Directiva General / Coordinación Regional</t>
+        </is>
+      </c>
+      <c r="G2" s="25" t="inlineStr">
+        <is>
+          <t>Electo y Juramentado</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Vicepresidenta</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Dra. Marlen Calvo Solano</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>2026 – 2028</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>Doctora en Enfermería / Académica</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>Comité de Educación y Asuntos Académicos</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Electa y Juramentada</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Secretaria General</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Dra. Patricia Quesada Steller</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>2026 – 2028</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Especialista en Enfermería</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>Secretaría de Actas y Archivo Oficial</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>Electa y Juramentada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Tesorero</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Dr. Josué Paniagua Sánchez</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>2026 – 2028</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>Especialista en Enfermería</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>Tesorería y Gestión Financiera</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Electo y Juramentado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Fiscal</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Dra. Janet Morales Salazar</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>2026 – 2028</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Especialista en Enfermería</t>
+        </is>
+      </c>
+      <c r="E6" s="25" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Fiscalía Deontológica y Estatutaria</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>Electa y Juramentada</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Vocal 1</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Dr. Marco Antonio Obando Rodríguez</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>2026 – 2028</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Especialista en Enfermería</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>Vocalía I / Enlace Institucional</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Electo y Juramentado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Vocal 2</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Dr. Fibier Olmos Venegas</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>2026 – 2028</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Especialista en Enfermería</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Vocalía II / Apoyo Operativo Regional</t>
+        </is>
+      </c>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>Electo y Juramentado</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1422,7 +1763,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1578,7 +1919,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat: asignar a Dra. Janet Morales Salazar como Fiscal en Junta Directiva y Acta Fundacional
</commit_message>
<xml_diff>
--- a/Directorio_ARCCPCE_Oficial.xlsx
+++ b/Directorio_ARCCPCE_Oficial.xlsx
@@ -1568,12 +1568,12 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Socia Fundadora</t>
+          <t>Fiscal de la Junta Directiva (2026-2028)</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>Asamblea General Constituyente</t>
+          <t>Junta Directiva General / Fiscalía Deontológica</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="I13" s="20" t="inlineStr">
         <is>
-          <t>Socia Fundadora Oficial</t>
+          <t>Activo - Junta Directiva (Fiscal)</t>
         </is>
       </c>
       <c r="J13" s="21" t="inlineStr">

</xml_diff>

<commit_message>
feat(hub): incorporar representacion oficial de Guatemala (Dra. Karen Dubon y Lic. Leticia De Aguinaga) y depurar contactos institucionales en mapas
</commit_message>
<xml_diff>
--- a/Directorio_ARCCPCE_Oficial.xlsx
+++ b/Directorio_ARCCPCE_Oficial.xlsx
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1755,6 +1755,110 @@
       <c r="J16" s="17" t="inlineStr">
         <is>
           <t>Acta Constitutiva (San José, 19-03-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>ARCCPCE-GT-001</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Dra. Karen Lorena Dubon De Paz</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>Representante Oficial de Guatemala</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>Delegación Nacional Guatemala</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>Doctorado / Maestría en Enfermería</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>Educación Médica, Simulación y Salud Pública</t>
+        </is>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>Delegación ARCCPCE Guatemala</t>
+        </is>
+      </c>
+      <c r="I17" s="20" t="inlineStr">
+        <is>
+          <t>Activa - Delegación Oficial</t>
+        </is>
+      </c>
+      <c r="J17" s="21" t="inlineStr">
+        <is>
+          <t>Acreditación Regional ARCCPCE (2026-2028)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>ARCCPCE-GT-002</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Lic. Leticia De Aguinaga</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Representante Oficial de Guatemala</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Delegación Nacional Guatemala</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Licenciatura en Enfermería</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>Gestión Gremial y Práctica Clínica</t>
+        </is>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>Delegación ARCCPCE Guatemala</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>Activa - Delegación Oficial</t>
+        </is>
+      </c>
+      <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>Acreditación Regional ARCCPCE (2026-2028)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(hub): incorporar a Mag. Cruz Barahona como representacion oficial de El Salvador
</commit_message>
<xml_diff>
--- a/Directorio_ARCCPCE_Oficial.xlsx
+++ b/Directorio_ARCCPCE_Oficial.xlsx
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1857,6 +1857,58 @@
         </is>
       </c>
       <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>Acreditación Regional ARCCPCE (2026-2028)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>ARCCPCE-SV-001</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Mag. Cruz Barahona</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>El Salvador</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>Representante Oficial de El Salvador</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>Delegación Nacional El Salvador</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>Magíster en Enfermería / Especialista</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="inlineStr">
+        <is>
+          <t>Cuidados Críticos, Gestión en Salud y Práctica Avanzada</t>
+        </is>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>Delegación ARCCPCE El Salvador</t>
+        </is>
+      </c>
+      <c r="I19" s="20" t="inlineStr">
+        <is>
+          <t>Activo - Delegación Oficial</t>
+        </is>
+      </c>
+      <c r="J19" s="21" t="inlineStr">
         <is>
           <t>Acreditación Regional ARCCPCE (2026-2028)</t>
         </is>

</xml_diff>

<commit_message>
feat(hub): incorporar a Mag. Orbelia Lopez como representacion oficial de Honduras
</commit_message>
<xml_diff>
--- a/Directorio_ARCCPCE_Oficial.xlsx
+++ b/Directorio_ARCCPCE_Oficial.xlsx
@@ -53,7 +53,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -106,6 +106,12 @@
         <bgColor rgb="00F0F7FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+        <bgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -147,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -225,6 +231,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -911,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1911,6 +1926,58 @@
       <c r="J19" s="21" t="inlineStr">
         <is>
           <t>Acreditación Regional ARCCPCE (2026-2028)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>ARCCPCE-HN-001</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>Mag. Orbelia López</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Honduras</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>Representante Oficial de Honduras</t>
+        </is>
+      </c>
+      <c r="E20" s="29" t="inlineStr">
+        <is>
+          <t>Comité de Salud Pública y Gestión Comunitaria</t>
+        </is>
+      </c>
+      <c r="F20" s="29" t="inlineStr">
+        <is>
+          <t>Magíster en Enfermería / Salud Pública</t>
+        </is>
+      </c>
+      <c r="G20" s="29" t="inlineStr">
+        <is>
+          <t>Salud Pública &amp; APS Comunitaria</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="inlineStr">
+        <is>
+          <t>Colegio de Profesionales de Enfermería de Honduras</t>
+        </is>
+      </c>
+      <c r="I20" s="29" t="inlineStr">
+        <is>
+          <t>Activo - Delegación Oficial</t>
+        </is>
+      </c>
+      <c r="J20" s="29" t="inlineStr">
+        <is>
+          <t>Nombramiento Institucional Oficial ARCCPCE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(governance): ajustar vocalias oficiales - Dr. Fibier Olmos Venegas como Vocal 1 y Dr. Marco Antonio Obando Rodriguez como Vocal 2
</commit_message>
<xml_diff>
--- a/Directorio_ARCCPCE_Oficial.xlsx
+++ b/Directorio_ARCCPCE_Oficial.xlsx
@@ -849,7 +849,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Dr. Marco Antonio Obando Rodríguez</t>
+          <t>Dr. Fibier Olmos Venegas</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>Dr. Fibier Olmos Venegas</t>
+          <t>Dr. Marco Antonio Obando Rodríguez</t>
         </is>
       </c>
       <c r="C8" s="25" t="inlineStr">

</xml_diff>